<commit_message>
D3 feedback round 2: space checks, long goods, small parts, own KPIs
- Loose containers: zone sized on 568 receipts (91% fit); big containers
  borrow the north half of receiving by blocking door R2 (97% fit).
- Outbound staging (216 m2) and packing (450 m2) validated on measured data.
- Max real length 2.05 m (longer WMS lengths are data errors); long-goods
  module with 4.5 m bays behind a 3.2 m aisle (VDI Ast check, load centre).
- Small slow parts move from pallet locations to bin shelving next to the
  put-wall (frees 1,005 locations); Kardex lifts compared as upgrade path.
- Own design KPIs, labour EUR 20/h, process-only payback, hazmat recount and
  classification by customs code (mostly PGS 37-2).
- Registers A042-A045 and S026-S030; D1/D2/D3, workbook and renders rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019BDu8Mejto8wmgVTUqspvV
</commit_message>
<xml_diff>
--- a/deliverables/Deliverable_3_Calculations.xlsx
+++ b/deliverables/Deliverable_3_Calculations.xlsx
@@ -15,8 +15,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPEX" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labour" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPIs" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stress test" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Small parts" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stress test" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="labour_rate">'Inputs'!$B$2</definedName>
@@ -26,31 +27,35 @@
     <definedName name="days_year">'Inputs'!$B$6</definedName>
     <definedName name="indirect_fte">'Inputs'!$B$7</definedName>
     <definedName name="rack_pp">'Inputs'!$B$8</definedName>
-    <definedName name="cantilever_pp">'Inputs'!$B$9</definedName>
-    <definedName name="rack_reuse">'Inputs'!$B$10</definedName>
-    <definedName name="rack_protect">'Inputs'!$B$11</definedName>
-    <definedName name="flow_bay">'Inputs'!$B$12</definedName>
-    <definedName name="ptl_slot">'Inputs'!$B$13</definedName>
-    <definedName name="ptl_integr">'Inputs'!$B$14</definedName>
-    <definedName name="rf_unit">'Inputs'!$B$15</definedName>
-    <definedName name="pack_station">'Inputs'!$B$16</definedName>
-    <definedName name="trolley">'Inputs'!$B$17</definedName>
-    <definedName name="tote">'Inputs'!$B$18</definedName>
-    <definedName name="wrapper">'Inputs'!$B$19</definedName>
-    <definedName name="conveyor">'Inputs'!$B$20</definedName>
-    <definedName name="roll_cage">'Inputs'!$B$21</definedName>
-    <definedName name="wms_config">'Inputs'!$B$22</definedName>
-    <definedName name="contingency">'Inputs'!$B$23</definedName>
-    <definedName name="lease_etv">'Inputs'!$B$24</definedName>
-    <definedName name="lease_eje">'Inputs'!$B$25</definedName>
-    <definedName name="lease_ere">'Inputs'!$B$26</definedName>
-    <definedName name="kwh_truck_h">'Inputs'!$B$27</definedName>
-    <definedName name="power_price">'Inputs'!$B$28</definedName>
-    <definedName name="rack_inspect">'Inputs'!$B$29</definedName>
-    <definedName name="it_support">'Inputs'!$B$30</definedName>
-    <definedName name="life_rack">'Inputs'!$B$31</definedName>
-    <definedName name="life_equip">'Inputs'!$B$32</definedName>
-    <definedName name="life_it">'Inputs'!$B$33</definedName>
+    <definedName name="long_bay_pp">'Inputs'!$B$9</definedName>
+    <definedName name="shelf_bay">'Inputs'!$B$10</definedName>
+    <definedName name="vlm_unit">'Inputs'!$B$11</definedName>
+    <definedName name="vlm_slot">'Inputs'!$B$12</definedName>
+    <definedName name="vlm_integr">'Inputs'!$B$13</definedName>
+    <definedName name="rack_reuse">'Inputs'!$B$14</definedName>
+    <definedName name="rack_protect">'Inputs'!$B$15</definedName>
+    <definedName name="flow_bay">'Inputs'!$B$16</definedName>
+    <definedName name="ptl_slot">'Inputs'!$B$17</definedName>
+    <definedName name="ptl_integr">'Inputs'!$B$18</definedName>
+    <definedName name="rf_unit">'Inputs'!$B$19</definedName>
+    <definedName name="pack_station">'Inputs'!$B$20</definedName>
+    <definedName name="trolley">'Inputs'!$B$21</definedName>
+    <definedName name="tote">'Inputs'!$B$22</definedName>
+    <definedName name="wrapper">'Inputs'!$B$23</definedName>
+    <definedName name="conveyor">'Inputs'!$B$24</definedName>
+    <definedName name="roll_cage">'Inputs'!$B$25</definedName>
+    <definedName name="wms_config">'Inputs'!$B$26</definedName>
+    <definedName name="contingency">'Inputs'!$B$27</definedName>
+    <definedName name="lease_etv">'Inputs'!$B$28</definedName>
+    <definedName name="lease_eje">'Inputs'!$B$29</definedName>
+    <definedName name="lease_ere">'Inputs'!$B$30</definedName>
+    <definedName name="kwh_truck_h">'Inputs'!$B$31</definedName>
+    <definedName name="power_price">'Inputs'!$B$32</definedName>
+    <definedName name="rack_inspect">'Inputs'!$B$33</definedName>
+    <definedName name="it_support">'Inputs'!$B$34</definedName>
+    <definedName name="life_rack">'Inputs'!$B$35</definedName>
+    <definedName name="life_equip">'Inputs'!$B$36</definedName>
+    <definedName name="life_it">'Inputs'!$B$37</definedName>
     <definedName name="dir_h_day">'Volumes'!$B$2</definedName>
     <definedName name="loose_crew">'Volumes'!$B$3</definedName>
     <definedName name="loose_h_cont">'Volumes'!$B$4</definedName>
@@ -59,18 +64,20 @@
     <definedName name="orders_day">'Volumes'!$B$7</definedName>
     <definedName name="inb_day">'Volumes'!$B$8</definedName>
     <definedName name="positions">'Volumes'!$B$9</definedName>
-    <definedName name="n_etv">'Volumes'!$B$10</definedName>
-    <definedName name="n_eje">'Volumes'!$B$11</definedName>
-    <definedName name="n_ere">'Volumes'!$B$12</definedName>
-    <definedName name="etv_h_day">'Volumes'!$B$13</definedName>
-    <definedName name="pt_h_day">'Volumes'!$B$14</definedName>
-    <definedName name="t_put_min">'Volumes'!$B$15</definedName>
-    <definedName name="loads_now">'Volumes'!$B$16</definedName>
-    <definedName name="pick_today_h">'Volumes'!$B$17</definedName>
-    <definedName name="pick_future_h">'Volumes'!$B$18</definedName>
-    <definedName name="capex_total">'CAPEX'!$F$19</definedName>
-    <definedName name="depreciation">'CAPEX'!$H$19</definedName>
-    <definedName name="capex_reuse">'CAPEX'!$F$21</definedName>
+    <definedName name="positions_long">'Volumes'!$B$10</definedName>
+    <definedName name="n_etv">'Volumes'!$B$11</definedName>
+    <definedName name="n_eje">'Volumes'!$B$12</definedName>
+    <definedName name="n_ere">'Volumes'!$B$13</definedName>
+    <definedName name="etv_h_day">'Volumes'!$B$14</definedName>
+    <definedName name="pt_h_day">'Volumes'!$B$15</definedName>
+    <definedName name="t_put_min">'Volumes'!$B$16</definedName>
+    <definedName name="loads_now">'Volumes'!$B$17</definedName>
+    <definedName name="pick_today_h">'Volumes'!$B$18</definedName>
+    <definedName name="pick_future_h">'Volumes'!$B$19</definedName>
+    <definedName name="capex_total">'CAPEX'!$F$21</definedName>
+    <definedName name="depreciation">'CAPEX'!$H$21</definedName>
+    <definedName name="capex_reuse">'CAPEX'!$F$23</definedName>
+    <definedName name="capex_process">'CAPEX'!$F$24</definedName>
     <definedName name="opex_total">'OPEX'!$F$11</definedName>
     <definedName name="loose_cost_year">'OPEX'!$F$3</definedName>
     <definedName name="labour_rows">'OPEX'!$F$2:$F$4</definedName>
@@ -579,7 +586,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Sheets: Inputs · Volumes · CAPEX · OPEX · Summary · Labour · KPIs · Stress test · Sensitivity</t>
+          <t>Sheets: Summary · Inputs · Volumes · CAPEX · OPEX · Labour · KPIs · Small parts · Stress test · Sensitivity</t>
         </is>
       </c>
     </row>
@@ -589,6 +596,166 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Direct FTE (peak day)</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>ETV 216i needed</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>EJE 120i needed</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>ERE 225 needed</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Outbound doors (busiest hour)</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Pickers in the busiest wave</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>150%</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>200%</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>250%</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -632,10 +799,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>580547</v>
+        <v>470905</v>
       </c>
       <c r="C2" t="n">
-        <v>605867</v>
+        <v>496225</v>
       </c>
       <c r="D2" t="n">
         <v>25320</v>
@@ -644,49 +811,49 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Racking price (€80–200/position)</t>
+          <t>Productivity ±20% (labour hours)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>553677</v>
+        <v>443980</v>
       </c>
       <c r="C3" t="n">
-        <v>641494</v>
+        <v>517271</v>
       </c>
       <c r="D3" t="n">
-        <v>87817</v>
+        <v>73291</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Productivity ±20% (labour hours)</t>
+          <t>Racking price (€80–200/position)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>539401</v>
+        <v>446129</v>
       </c>
       <c r="C4" t="n">
-        <v>641134</v>
+        <v>528920</v>
       </c>
       <c r="D4" t="n">
-        <v>101733</v>
+        <v>82790</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Labour rate (€24–34/h)</t>
+          <t>Labour rate (€20–28/h)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>547688</v>
+        <v>480625</v>
       </c>
       <c r="C5" t="n">
-        <v>654137</v>
+        <v>566409</v>
       </c>
       <c r="D5" t="n">
-        <v>106449</v>
+        <v>85784</v>
       </c>
     </row>
   </sheetData>
@@ -700,7 +867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -936,14 +1103,30 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>Payback, process changes only (years)</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>capex_process/B12</f>
+        <v/>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>process CAPEX ÷ saving</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
           <t>Loose container: in-house cost per container</t>
         </is>
       </c>
-      <c r="B15" s="5">
+      <c r="B16" s="5">
         <f>loose_cost_year/(cont_day*days_year)</f>
         <v/>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>break-even price for a contractor</t>
         </is>
@@ -960,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1016,14 +1199,14 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2" t="n">
         <v>28</v>
       </c>
-      <c r="C2" t="n">
-        <v>24</v>
-      </c>
-      <c r="D2" t="n">
-        <v>34</v>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>EUR per paid hour (operative)</t>
@@ -1036,7 +1219,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CAO Beroepsgoederenvervoer 2025 wage scales B-C EUR 14.40-18.28/h (S019) x 1.08 holiday pay x 1.33 employer premiums (CBS transport &amp; storage: EUR 10.9 premiums on EUR 33.5 wages per worked hour, S018) x 1.19 paid-but-not-worked time; stays below the CBS sector average of EUR 44.4 (which includes drivers and managers)</t>
+          <t>teacher feedback (S026): EUR 20/h for a warehouse operator; high end EUR 28/h = CAO wage (S019) x employer premiums (S018) x holiday pay x paid-not-worked time</t>
         </is>
       </c>
     </row>
@@ -1047,14 +1230,14 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="C3" t="n">
+        <v>27</v>
+      </c>
+      <c r="D3" t="n">
         <v>38</v>
       </c>
-      <c r="C3" t="n">
-        <v>32</v>
-      </c>
-      <c r="D3" t="n">
-        <v>45</v>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>EUR per paid hour (team leader)</t>
@@ -1067,7 +1250,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CAO scale F-G EUR 23-25/h (S019) x same factors</t>
+          <t>operator rate x 1.35 (CAO scale F-G vs B-C, S019)</t>
         </is>
       </c>
     </row>
@@ -1078,14 +1261,14 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D4" t="n">
         <v>33</v>
       </c>
-      <c r="C4" t="n">
-        <v>28</v>
-      </c>
-      <c r="D4" t="n">
-        <v>40</v>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>EUR per paid hour (inventory control / admin)</t>
@@ -1098,7 +1281,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>between operative and team leader</t>
+          <t>operator rate x 1.2</t>
         </is>
       </c>
     </row>
@@ -1229,21 +1412,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cantilever_pp</t>
+          <t>long_bay_pp</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
+        <v>160</v>
+      </c>
+      <c r="C9" t="n">
+        <v>100</v>
+      </c>
+      <c r="D9" t="n">
         <v>250</v>
       </c>
-      <c r="C9" t="n">
-        <v>150</v>
-      </c>
-      <c r="D9" t="n">
-        <v>400</v>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>EUR per arm position</t>
+          <t>EUR per long-goods position (4.5 m beams)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1253,307 +1436,307 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>assumption: ~2x a pallet position (heavier column + arms)</t>
+          <t>assumption: ~1.25x a standard position (longer, heavier beams)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rack_reuse</t>
+          <t>shelf_bay</t>
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>25</v>
+        <v>200</v>
       </c>
       <c r="C10" t="n">
-        <v>15</v>
+        <v>153</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>245</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>EUR per position to dismantle + re-assemble existing racking</t>
+          <t>EUR per bin-shelving bay (1.0 x 0.6 x 2.5 m)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>A033</t>
+          <t>A042</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>assumption: ~20% of a new installed position; only if today's racking fits the new layout (to confirm with DHL)</t>
+          <t>Manutan shelving EUR 153-245 per section (S030)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>rack_protect</t>
+          <t>vlm_unit</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>0.05</v>
+        <v>60000</v>
       </c>
       <c r="C11" t="n">
-        <v>0.03</v>
+        <v>48000</v>
       </c>
       <c r="D11" t="n">
-        <v>0.08</v>
+        <v>90000</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>share of racking cost</t>
+          <t>EUR per Kardex Shuttle XP 500 incl. installation (compared option)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>A033</t>
+          <t>A042</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>end-of-aisle guards, upright protectors, load signs (EN 15635, S015)</t>
+          <t>new Shuttle XP 500 (2,450 x 864 trays) EUR 48,000 (S027); 4,050 mm trays + installation -&gt; EUR 60,000 assumed</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>flow_bay</t>
+          <t>vlm_slot</t>
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>1800</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
-        <v>1100</v>
+        <v>6</v>
       </c>
       <c r="D12" t="n">
-        <v>2300</v>
+        <v>12</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>EUR per carton-flow bay (2 m, 5 levels)</t>
+          <t>EUR per half-bin slot (bin + divider)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>A034</t>
+          <t>A042</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>new USD 1,200-2,500 per bay (S025) at ~0.9 EUR/USD; used EUR 650/bay (S025) = floor</t>
+          <t>half of a 600x400 tote EUR 14.56-19.95 (S025)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ptl_slot</t>
+          <t>vlm_integr</t>
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>150</v>
+        <v>10000</v>
       </c>
       <c r="C13" t="n">
-        <v>60</v>
+        <v>5000</v>
       </c>
       <c r="D13" t="n">
-        <v>200</v>
+        <v>20000</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>EUR per put-to-light slot</t>
+          <t>EUR one-off</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>A035</t>
+          <t>A042</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>USD 60-200 per station (S025)</t>
+          <t>assumption: WMS link to the lift controller + light pointer</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ptl_integr</t>
+          <t>rack_reuse</t>
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>12000</v>
+        <v>25</v>
       </c>
       <c r="C14" t="n">
-        <v>5000</v>
+        <v>15</v>
       </c>
       <c r="D14" t="n">
-        <v>30000</v>
+        <v>40</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>EUR one-off</t>
+          <t>EUR per position to dismantle + re-assemble existing racking</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>A035</t>
+          <t>A033</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>installation + WMS integration USD 3,000-18,000 + software (S025)</t>
+          <t>assumption: ~20% of a new installed position; only if today's racking fits the new layout (to confirm with DHL)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rf_unit</t>
+          <t>rack_protect</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>1500</v>
+        <v>0.05</v>
       </c>
       <c r="C15" t="n">
-        <v>450</v>
+        <v>0.03</v>
       </c>
       <c r="D15" t="n">
-        <v>2300</v>
+        <v>0.08</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>EUR per RF terminal incl. cradle</t>
+          <t>share of racking cost</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>A036</t>
+          <t>A033</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Zebra MC3300 listings EUR 435-2,326 + cradle EUR 182 (S025)</t>
+          <t>end-of-aisle guards, upright protectors, load signs (EN 15635, S015)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>pack_station</t>
+          <t>flow_bay</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>2500</v>
+        <v>1800</v>
       </c>
       <c r="C16" t="n">
-        <v>1500</v>
+        <v>1100</v>
       </c>
       <c r="D16" t="n">
-        <v>4000</v>
+        <v>2300</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>EUR per pack station</t>
+          <t>EUR per carton-flow bay (2 m, 5 levels)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>A036</t>
+          <t>A034</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>assumption: bench, scale, label printer</t>
+          <t>new USD 1,200-2,500 per bay (S025) at ~0.9 EUR/USD; used EUR 650/bay (S025) = floor</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>trolley</t>
+          <t>ptl_slot</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>433</v>
+        <v>150</v>
       </c>
       <c r="C17" t="n">
-        <v>280</v>
+        <v>60</v>
       </c>
       <c r="D17" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>EUR per pick trolley</t>
+          <t>EUR per put-to-light slot</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>A036</t>
+          <t>A035</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Fetra picking trolley EUR 432.86 net (S025)</t>
+          <t>USD 60-200 per station (S025)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>tote</t>
+          <t>ptl_integr</t>
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>16</v>
+        <v>12000</v>
       </c>
       <c r="C18" t="n">
-        <v>14</v>
+        <v>5000</v>
       </c>
       <c r="D18" t="n">
-        <v>20</v>
+        <v>30000</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>EUR per tote 600x400x320</t>
+          <t>EUR one-off</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>A036</t>
+          <t>A035</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>EUR 14.56-19.95 (S025)</t>
+          <t>installation + WMS integration USD 3,000-18,000 + software (S025)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>wrapper</t>
+          <t>rf_unit</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>3849</v>
+        <v>1500</v>
       </c>
       <c r="C19" t="n">
-        <v>3000</v>
+        <v>450</v>
       </c>
       <c r="D19" t="n">
-        <v>9000</v>
+        <v>2300</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>EUR per semi-automatic stretch wrapper</t>
+          <t>EUR per RF terminal incl. cradle</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1563,28 +1746,28 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Vogel Starter EUR 3,849 new (S025)</t>
+          <t>Zebra MC3300 listings EUR 435-2,326 + cradle EUR 182 (S025)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>conveyor</t>
+          <t>pack_station</t>
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>1250</v>
+        <v>2500</v>
       </c>
       <c r="C20" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="D20" t="n">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>EUR per extendable roller conveyor (4.5 m)</t>
+          <t>EUR per pack station</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1594,28 +1777,28 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Cromwell GBP 1,049 ex VAT (S025)</t>
+          <t>assumption: bench, scale, label printer</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>roll_cage</t>
+          <t>trolley</t>
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>150</v>
+        <v>433</v>
       </c>
       <c r="C21" t="n">
-        <v>100</v>
+        <v>280</v>
       </c>
       <c r="D21" t="n">
-        <v>250</v>
+        <v>600</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>EUR per roll cage</t>
+          <t>EUR per pick trolley</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1625,107 +1808,107 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>Fetra picking trolley EUR 432.86 net (S025)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>wms_config</t>
+          <t>tote</t>
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>25000</v>
+        <v>16</v>
       </c>
       <c r="C22" t="n">
-        <v>10000</v>
+        <v>14</v>
       </c>
       <c r="D22" t="n">
-        <v>50000</v>
+        <v>20</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>EUR one-off</t>
+          <t>EUR per tote 600x400x320</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>A037</t>
+          <t>A036</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>assumption: WMS set-up of waves, put-wall, slotting &amp; putaway rules (~25 consultant days)</t>
+          <t>EUR 14.56-19.95 (S025)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>contingency</t>
+          <t>wrapper</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>0.1</v>
+        <v>3849</v>
       </c>
       <c r="C23" t="n">
-        <v>0.05</v>
+        <v>3000</v>
       </c>
       <c r="D23" t="n">
-        <v>0.2</v>
+        <v>9000</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>share of CAPEX</t>
+          <t>EUR per semi-automatic stretch wrapper</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>A037</t>
+          <t>A036</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>planning allowance</t>
+          <t>Vogel Starter EUR 3,849 new (S025)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lease_etv</t>
+          <t>conveyor</t>
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>900</v>
+        <v>1250</v>
       </c>
       <c r="C24" t="n">
-        <v>495</v>
+        <v>1000</v>
       </c>
       <c r="D24" t="n">
-        <v>1550</v>
+        <v>2500</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>EUR per month, full-service lease</t>
+          <t>EUR per extendable roller conveyor (4.5 m)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>A038</t>
+          <t>A036</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Dutch reach-truck lease offers EUR 350-495/month all-in (72 months) up to rental EUR 1,100-1,550/month (S021); 10.7 m Li-ion truck -&gt; upper half</t>
+          <t>Cromwell GBP 1,049 ex VAT (S025)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lease_eje</t>
+          <t>roll_cage</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
@@ -1739,263 +1922,387 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>EUR per month, full-service lease</t>
+          <t>EUR per roll cage</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>A038</t>
+          <t>A036</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>assumption: Li-ion pallet truck new ~EUR 2,500-3,500 (S025) over 72 months + service</t>
+          <t>assumption</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>lease_ere</t>
+          <t>wms_config</t>
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>350</v>
+        <v>25000</v>
       </c>
       <c r="C26" t="n">
-        <v>250</v>
+        <v>10000</v>
       </c>
       <c r="D26" t="n">
-        <v>500</v>
+        <v>50000</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>EUR per month, full-service lease</t>
+          <t>EUR one-off</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>A038</t>
+          <t>A037</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>assumption: rider pallet truck, between pallet truck and reach truck</t>
+          <t>assumption: WMS set-up of waves, put-wall, slotting &amp; putaway rules (~25 consultant days)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>kwh_truck_h</t>
+          <t>contingency</t>
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>4</v>
+        <v>0.1</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>0.05</v>
       </c>
       <c r="D27" t="n">
-        <v>6</v>
+        <v>0.2</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>kWh per truck operating hour (ETV); 1.5 for pallet trucks</t>
+          <t>share of CAPEX</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>A039</t>
+          <t>A037</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>assumption</t>
+          <t>planning allowance</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>power_price</t>
+          <t>lease_etv</t>
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>0.2046</v>
+        <v>900</v>
       </c>
       <c r="C28" t="n">
-        <v>0.17</v>
+        <v>495</v>
       </c>
       <c r="D28" t="n">
-        <v>0.25</v>
+        <v>1550</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>EUR per kWh</t>
+          <t>EUR per month, full-service lease</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>A039</t>
+          <t>A038</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Eurostat nrg_pc_205, NL non-household 500-2,000 MWh, H1 2025 (S022)</t>
+          <t>Dutch reach-truck lease offers EUR 350-495/month all-in (72 months) up to rental EUR 1,100-1,550/month (S021); 10.7 m Li-ion truck -&gt; upper half</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>rack_inspect</t>
+          <t>lease_eje</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>2500</v>
+        <v>150</v>
       </c>
       <c r="C29" t="n">
-        <v>1500</v>
+        <v>100</v>
       </c>
       <c r="D29" t="n">
-        <v>4000</v>
+        <v>250</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>EUR per year</t>
+          <t>EUR per month, full-service lease</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>A040</t>
+          <t>A038</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>assumption: 1 expert inspection per year (EN 15635, S015)</t>
+          <t>assumption: Li-ion pallet truck new ~EUR 2,500-3,500 (S025) over 72 months + service</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>it_support</t>
+          <t>lease_ere</t>
         </is>
       </c>
       <c r="B30" s="9" t="n">
-        <v>0.15</v>
+        <v>350</v>
       </c>
       <c r="C30" t="n">
-        <v>0.1</v>
+        <v>250</v>
       </c>
       <c r="D30" t="n">
-        <v>0.2</v>
+        <v>500</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>share of IT CAPEX per year</t>
+          <t>EUR per month, full-service lease</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>A040</t>
+          <t>A038</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>assumption: device repair, licences, spares</t>
+          <t>assumption: rider pallet truck, between pallet truck and reach truck</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>life_rack</t>
+          <t>kwh_truck_h</t>
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>kWh per truck operating hour (ETV); 1.5 for pallet trucks</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>A041</t>
+          <t>A039</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>straight-line depreciation</t>
+          <t>assumption</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>life_equip</t>
+          <t>power_price</t>
         </is>
       </c>
       <c r="B32" s="9" t="n">
-        <v>7</v>
+        <v>0.2046</v>
       </c>
       <c r="C32" t="n">
-        <v>7</v>
+        <v>0.17</v>
       </c>
       <c r="D32" t="n">
-        <v>7</v>
+        <v>0.25</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>EUR per kWh</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>A041</t>
+          <t>A039</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>straight-line depreciation</t>
+          <t>Eurostat nrg_pc_205, NL non-household 500-2,000 MWh, H1 2025 (S022)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>rack_inspect</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D33" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>EUR per year</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>A040</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>assumption: 1 expert inspection per year (EN 15635, S015)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>it_support</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>share of IT CAPEX per year</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>A040</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>assumption: device repair, licences, spares</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>life_rack</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="C35" t="n">
+        <v>15</v>
+      </c>
+      <c r="D35" t="n">
+        <v>15</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>A041</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>straight-line depreciation</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>life_equip</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="C36" t="n">
+        <v>7</v>
+      </c>
+      <c r="D36" t="n">
+        <v>7</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>A041</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>straight-line depreciation</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>life_it</t>
         </is>
       </c>
-      <c r="B33" s="9" t="n">
+      <c r="B37" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C37" t="n">
         <v>5</v>
       </c>
-      <c r="D33" t="n">
+      <c r="D37" t="n">
         <v>5</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>A041</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>straight-line depreciation</t>
         </is>
@@ -2012,7 +2319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2050,7 +2357,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>34.9</v>
+        <v>35.2</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -2190,11 +2497,11 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>9504</v>
+        <v>8960</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>pallet positions (single-deep)</t>
+          <t>pallet positions (single-deep, incl. long goods)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2206,55 +2513,55 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>n_etv</t>
+          <t>positions_long</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>2</v>
+        <v>320</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ETV 216i reach trucks</t>
+          <t>long-goods positions (4.5 m bays)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>fleet review (D3 §4)</t>
+          <t>floor plan</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>n_eje</t>
+          <t>n_etv</t>
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>EJE 120i pallet trucks</t>
+          <t>ETV 216i reach trucks</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>fleet review</t>
+          <t>fleet review (D3 §4)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>n_ere</t>
+          <t>n_eje</t>
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ERE 225 rider pallet trucks</t>
+          <t>EJE 120i pallet trucks</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2266,35 +2573,35 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>etv_h_day</t>
+          <t>n_ere</t>
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>4.9</v>
+        <v>2</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ETV operating hours per day</t>
+          <t>ERE 225 rider pallet trucks</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>cycle-time model</t>
+          <t>fleet review</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>pt_h_day</t>
+          <t>etv_h_day</t>
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>10</v>
+        <v>4.9</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>pallet-truck operating hours per day</t>
+          <t>ETV operating hours per day</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2306,15 +2613,15 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>t_put_min</t>
+          <t>pt_h_day</t>
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>2.38</v>
+        <v>9.100000000000001</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>putaway cycle, minutes per pallet</t>
+          <t>pallet-truck operating hours per day</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2326,58 +2633,78 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>loads_now</t>
+          <t>t_put_min</t>
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>11015</v>
+        <v>2.38</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>loads to move in once (re-slotting)</t>
+          <t>putaway cycle, minutes per pallet</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>measured</t>
+          <t>cycle-time model</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>pick_today_h</t>
+          <t>loads_now</t>
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>31.13</v>
+        <v>11015</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>picker-hours/day today (modelled, incl. 08:00 peak staffing)</t>
+          <t>loads to move in once (re-slotting)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>D3 §2.2</t>
+          <t>measured</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>pick_today_h</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>31.143</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>picker-hours/day today (modelled, incl. 08:00 peak staffing)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>D3 §2.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>pick_future_h</t>
         </is>
       </c>
-      <c r="B18" s="10" t="n">
-        <v>11.37</v>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="B19" s="10" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>picker-hours/day in the design</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>pick-time model</t>
         </is>
@@ -2394,7 +2721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2467,7 +2794,7 @@
         </is>
       </c>
       <c r="C2" s="11">
-        <f>positions</f>
+        <f>positions-positions_long</f>
         <v/>
       </c>
       <c r="D2" t="inlineStr">
@@ -2505,19 +2832,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cantilever racking for goods &gt; 2.4 m</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="n">
-        <v>40</v>
+          <t>Long-goods racking, 4.5 m bays (2.05 m pallets)</t>
+        </is>
+      </c>
+      <c r="C3" s="11">
+        <f>positions_long</f>
+        <v/>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>arm positions</t>
+          <t>positions</t>
         </is>
       </c>
       <c r="E3" s="12">
-        <f>cantilever_pp</f>
+        <f>long_bay_pp</f>
         <v/>
       </c>
       <c r="F3" s="13">
@@ -2582,16 +2910,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Picking</t>
+          <t>Small-item storage</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Carton-flow bays, fast-pick area</t>
+          <t>Bin shelving for small parts (next to the put-wall)</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>31</v>
+        <v>188</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -2599,7 +2927,7 @@
         </is>
       </c>
       <c r="E5" s="12">
-        <f>flow_bay</f>
+        <f>shelf_bay</f>
         <v/>
       </c>
       <c r="F5" s="13">
@@ -2616,31 +2944,31 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>A034 / S025</t>
+          <t>A042 / S030</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Picking</t>
+          <t>Small-item storage</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pick trolleys (3-tier, 6 totes)</t>
+          <t>Half-bins and dividers</t>
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>6</v>
+        <v>3948</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>trolleys</t>
+          <t>slots</t>
         </is>
       </c>
       <c r="E6" s="12">
-        <f>trolley</f>
+        <f>vlm_slot</f>
         <v/>
       </c>
       <c r="F6" s="13">
@@ -2657,7 +2985,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>S011 / S025</t>
+          <t>A042 / S025</t>
         </is>
       </c>
     </row>
@@ -2669,19 +2997,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Totes 600 x 400</t>
+          <t>Carton-flow bays, fast-pick area</t>
         </is>
       </c>
       <c r="C7" s="11" t="n">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>totes</t>
+          <t>bays</t>
         </is>
       </c>
       <c r="E7" s="12">
-        <f>tote</f>
+        <f>flow_bay</f>
         <v/>
       </c>
       <c r="F7" s="13">
@@ -2698,31 +3026,31 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>S025</t>
+          <t>A034 / S025</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sorting &amp; packing</t>
+          <t>Picking</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Put-to-light wall (slots)</t>
+          <t>Pick trolleys (3-tier, 6 totes)</t>
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>90</v>
+        <v>6</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>slots</t>
+          <t>trolleys</t>
         </is>
       </c>
       <c r="E8" s="12">
-        <f>ptl_slot</f>
+        <f>trolley</f>
         <v/>
       </c>
       <c r="F8" s="13">
@@ -2739,31 +3067,31 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>A035 / S025</t>
+          <t>S011 / S025</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sorting &amp; packing</t>
+          <t>Picking</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Put-to-light installation + WMS link</t>
+          <t>Totes 600 x 400</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>totes</t>
         </is>
       </c>
       <c r="E9" s="12">
-        <f>ptl_integr</f>
+        <f>tote</f>
         <v/>
       </c>
       <c r="F9" s="13">
@@ -2780,7 +3108,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>A035 / S025</t>
+          <t>S025</t>
         </is>
       </c>
     </row>
@@ -2792,19 +3120,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pack stations (bench, scale, label printer)</t>
+          <t>Put-to-light wall (slots)</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>stations</t>
+          <t>slots</t>
         </is>
       </c>
       <c r="E10" s="12">
-        <f>pack_station</f>
+        <f>ptl_slot</f>
         <v/>
       </c>
       <c r="F10" s="13">
@@ -2821,7 +3149,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>A036</t>
+          <t>A035 / S025</t>
         </is>
       </c>
     </row>
@@ -2833,7 +3161,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Stretch wrapper (packing)</t>
+          <t>Put-to-light installation + WMS link</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
@@ -2841,11 +3169,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="E11" s="12">
-        <f>wrapper</f>
+        <f>ptl_integr</f>
         <v/>
       </c>
       <c r="F11" s="13">
@@ -2862,7 +3190,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>S025</t>
+          <t>A035 / S025</t>
         </is>
       </c>
     </row>
@@ -2874,19 +3202,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Roll cages for parcels</t>
+          <t>Pack stations (bench, scale, label printer)</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>41</v>
+        <v>4</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>cages</t>
+          <t>stations</t>
         </is>
       </c>
       <c r="E12" s="12">
-        <f>roll_cage</f>
+        <f>pack_station</f>
         <v/>
       </c>
       <c r="F12" s="13">
@@ -2910,16 +3238,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Loose-container zone</t>
+          <t>Sorting &amp; packing</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Extendable roller conveyor (into the container)</t>
+          <t>Stretch wrapper (packing)</t>
         </is>
       </c>
       <c r="C13" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -2927,7 +3255,7 @@
         </is>
       </c>
       <c r="E13" s="12">
-        <f>conveyor</f>
+        <f>wrapper</f>
         <v/>
       </c>
       <c r="F13" s="13">
@@ -2951,24 +3279,24 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Loose-container zone</t>
+          <t>Sorting &amp; packing</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Stretch wrapper (newly built pallets)</t>
+          <t>Roll cages for parcels</t>
         </is>
       </c>
       <c r="C14" s="11" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>cages</t>
         </is>
       </c>
       <c r="E14" s="12">
-        <f>wrapper</f>
+        <f>roll_cage</f>
         <v/>
       </c>
       <c r="F14" s="13">
@@ -2985,23 +3313,23 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>S025</t>
+          <t>A036</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Loose-container zone</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RF terminals with cradles</t>
+          <t>Extendable roller conveyor (into the container)</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -3009,7 +3337,7 @@
         </is>
       </c>
       <c r="E15" s="12">
-        <f>rf_unit</f>
+        <f>conveyor</f>
         <v/>
       </c>
       <c r="F15" s="13">
@@ -3017,7 +3345,7 @@
         <v/>
       </c>
       <c r="G15">
-        <f>life_it</f>
+        <f>life_equip</f>
         <v/>
       </c>
       <c r="H15" s="13">
@@ -3026,19 +3354,19 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>A036 / S025</t>
+          <t>S025</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Loose-container zone</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>WMS set-up: waves, put-wall, slotting, putaway rules</t>
+          <t>Stretch wrapper (newly built pallets)</t>
         </is>
       </c>
       <c r="C16" s="11" t="n">
@@ -3046,11 +3374,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>units</t>
         </is>
       </c>
       <c r="E16" s="12">
-        <f>wms_config</f>
+        <f>wrapper</f>
         <v/>
       </c>
       <c r="F16" s="13">
@@ -3058,7 +3386,7 @@
         <v/>
       </c>
       <c r="G16">
-        <f>life_it</f>
+        <f>life_equip</f>
         <v/>
       </c>
       <c r="H16" s="13">
@@ -3067,31 +3395,31 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>A037</t>
+          <t>S025</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>One-off</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Move-in / re-slotting (each load moved once)</t>
+          <t>RF terminals with cradles</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>11015</v>
+        <v>14</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>loads</t>
+          <t>units</t>
         </is>
       </c>
       <c r="E17" s="12">
-        <f>t_put_min/60*(labour_rate+lease_etv*12/(days_year*7.5))</f>
+        <f>rf_unit</f>
         <v/>
       </c>
       <c r="F17" s="13">
@@ -3099,7 +3427,7 @@
         <v/>
       </c>
       <c r="G17">
-        <f>life_equip</f>
+        <f>life_it</f>
         <v/>
       </c>
       <c r="H17" s="13">
@@ -3108,22 +3436,22 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>ETV cycle model + A030</t>
+          <t>A036 / S025</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Contingency</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Contingency on all items above</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
+          <t>WMS set-up: waves, put-wall, slotting, putaway rules</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
         <v>1</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -3131,8 +3459,8 @@
           <t>lot</t>
         </is>
       </c>
-      <c r="E18" s="13">
-        <f>contingency*SUM(F2:F17)</f>
+      <c r="E18" s="12">
+        <f>wms_config</f>
         <v/>
       </c>
       <c r="F18" s="13">
@@ -3140,7 +3468,7 @@
         <v/>
       </c>
       <c r="G18">
-        <f>life_equip</f>
+        <f>life_it</f>
         <v/>
       </c>
       <c r="H18" s="13">
@@ -3154,43 +3482,143 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="n"/>
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>TOTAL CAPEX</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="14" t="n"/>
-      <c r="E19" s="14" t="n"/>
-      <c r="F19" s="5">
-        <f>SUM(F2:F18)</f>
-        <v/>
-      </c>
-      <c r="G19" s="14" t="n"/>
-      <c r="H19" s="5">
-        <f>SUM(H2:H18)</f>
-        <v/>
-      </c>
-      <c r="I19" s="14" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>One-off</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Move-in / re-slotting (each load moved once)</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>11015</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>loads</t>
+        </is>
+      </c>
+      <c r="E19" s="12">
+        <f>t_put_min/60*(labour_rate+lease_etv*12/(days_year*7.5))</f>
+        <v/>
+      </c>
+      <c r="F19" s="13">
+        <f>C19*E19</f>
+        <v/>
+      </c>
+      <c r="G19">
+        <f>life_equip</f>
+        <v/>
+      </c>
+      <c r="H19" s="13">
+        <f>F19/G19</f>
+        <v/>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>ETV cycle model + A030</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Contingency on all items above</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="E20" s="13">
+        <f>contingency*SUM(F2:F19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="13">
+        <f>C20*E20</f>
+        <v/>
+      </c>
+      <c r="G20">
+        <f>life_equip</f>
+        <v/>
+      </c>
+      <c r="H20" s="13">
+        <f>F20/G20</f>
+        <v/>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>A037</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="n"/>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>CAPEX if today's racking is re-used (dismantle + rebuild at rack_reuse per position)</t>
+          <t>TOTAL CAPEX</t>
         </is>
       </c>
       <c r="C21" s="14" t="n"/>
       <c r="D21" s="14" t="n"/>
       <c r="E21" s="14" t="n"/>
       <c r="F21" s="5">
-        <f>(SUM(F2:F17)-F2-F4+positions*rack_reuse)*(1+contingency)</f>
+        <f>SUM(F2:F20)</f>
         <v/>
       </c>
       <c r="G21" s="14" t="n"/>
-      <c r="H21" s="14" t="n"/>
+      <c r="H21" s="5">
+        <f>SUM(H2:H20)</f>
+        <v/>
+      </c>
       <c r="I21" s="14" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="n"/>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>CAPEX if today's racking is re-used (dismantle + rebuild at rack_reuse per position)</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="14" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="5">
+        <f>(SUM(F2:F19)-F2-F3-F4+positions*rack_reuse)*(1+contingency)</f>
+        <v/>
+      </c>
+      <c r="G23" s="14" t="n"/>
+      <c r="H23" s="14" t="n"/>
+      <c r="I23" s="14" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="n"/>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>CAPEX of the process changes only (fast-pick, trolleys, totes, put-wall, RF, WMS set-up)</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="5">
+        <f>(F7+F8+F9+F10+F11+F17+F18)*(1+contingency)</f>
+        <v/>
+      </c>
+      <c r="G24" s="14" t="n"/>
+      <c r="H24" s="14" t="n"/>
+      <c r="I24" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3583,7 +4011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3803,7 +4231,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3819,16 +4247,16 @@
         <v>1.83</v>
       </c>
       <c r="F6" t="n">
-        <v>3.6</v>
+        <v>2.9</v>
       </c>
       <c r="G6" t="n">
-        <v>6.5</v>
+        <v>5.3</v>
       </c>
       <c r="H6" t="n">
-        <v>0.48</v>
+        <v>0.39</v>
       </c>
       <c r="I6" t="n">
-        <v>0.87</v>
+        <v>0.71</v>
       </c>
       <c r="J6" t="b">
         <v>1</v>
@@ -3841,7 +4269,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -3857,16 +4285,16 @@
         <v>1.83</v>
       </c>
       <c r="F7" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="G7" t="n">
-        <v>14.3</v>
+        <v>12.7</v>
       </c>
       <c r="H7" t="n">
-        <v>1.04</v>
+        <v>0.92</v>
       </c>
       <c r="I7" t="n">
-        <v>1.9</v>
+        <v>1.69</v>
       </c>
       <c r="J7" t="b">
         <v>1</v>
@@ -3875,34 +4303,36 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Full-pallet picking (reach truck)</t>
+          <t>Picking - small parts (bin shelving)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.4</v>
+        <v>1.9</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>pallets</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>22</v>
+          <t>picker-h</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="E8" t="n">
         <v>1.83</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3</v>
+        <v>1.9</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5</v>
+        <v>3.4</v>
       </c>
       <c r="H8" t="n">
-        <v>0.04</v>
+        <v>0.25</v>
       </c>
       <c r="I8" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.46</v>
       </c>
       <c r="J8" t="b">
         <v>1</v>
@@ -3911,34 +4341,34 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Packing / consolidation</t>
+          <t>Full-pallet picking (reach truck)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>633.6</v>
+        <v>6.4</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>lines</t>
+          <t>pallets</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="E9" t="n">
         <v>1.83</v>
       </c>
       <c r="F9" t="n">
-        <v>14.1</v>
+        <v>0.3</v>
       </c>
       <c r="G9" t="n">
-        <v>25.8</v>
+        <v>0.5</v>
       </c>
       <c r="H9" t="n">
-        <v>1.88</v>
+        <v>0.04</v>
       </c>
       <c r="I9" t="n">
-        <v>3.44</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="J9" t="b">
         <v>1</v>
@@ -3947,36 +4377,72 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Packing / consolidation</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>633.6</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>lines</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>45</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="F10" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Shipping / loading</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" t="n">
         <v>17.7</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>pallets</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>30</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E11" t="n">
         <v>2.85</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F11" t="n">
         <v>0.6</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G11" t="n">
         <v>1.7</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H11" t="n">
         <v>0.08</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I11" t="n">
         <v>0.22</v>
       </c>
-      <c r="J10" t="b">
+      <c r="J11" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3991,15 +4457,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4015,20 +4482,25 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>How it is measured</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Today (data)</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Future (design)</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Target / benchmark</t>
         </is>
@@ -4042,27 +4514,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pallet positions vs peak need</t>
+          <t>Rack fill at peak</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>positions provided / peak occupied locations</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8,512 occupied (peak)</t>
+          <t>pallet locations used at the peak ÷ rack positions</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>9,504 positions (90% full at peak, 85% on average)</t>
+          <t>8,512 locations used</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>≤ 90% full at peak (A010)</t>
+          <t>84% (7,507 of 8,960; small parts moved to bin shelving)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>≤ 90%</t>
         </is>
       </c>
     </row>
@@ -4074,27 +4551,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Floor area used</t>
+          <t>Storage headroom</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>zones + aisles / 7,000 m²</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>months until the racks are full at the Apr–Jun growth rate</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>6,731 m² (96%)</t>
+          <t>+10% locations in 2 months</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>≤ 7,000 m²</t>
+          <t>~4 months (~5 with a 12th module)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>≥ 12 months</t>
         </is>
       </c>
     </row>
@@ -4106,59 +4588,69 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Storage headroom</t>
+          <t>Small-item density</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>months until the racks are full if stock keeps growing as in Apr–Jun</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>+10% locations in 2 months</t>
+          <t>SKUs stored per m² of floor</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>~2 months</t>
+          <t>~2.6 SKUs/m² (one pallet location each)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>≥ 12 months → clear dead stock, add a 12th rack module</t>
+          <t>~13 SKUs/m² in bin shelving</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>≥ 5× better</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Inbound</t>
+          <t>Space</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dock-to-stock time</t>
+          <t>Floor area used</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>truck at the door → pallet in its location</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>large China receipts take 1–3 days to book in</t>
+          <t>zones + aisles ÷ 7,000 m²</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>~1.5 h per palletised trailer; ~3.8 h per loose container</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>&lt; 3.5 h best-in-class (S023)</t>
+          <t>6,731 m² (96%)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>≤ 7,000 m²</t>
         </is>
       </c>
     </row>
@@ -4170,313 +4662,363 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Put-away cycle time</t>
+          <t>Dock-to-stock time</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>minutes per pallet, reach truck</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>truck at the door → pallet in its location</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2.4 min per pallet (~25 per truck-hour)</t>
+          <t>big China receipts take 1–3 days to book in</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>≤ 3 min</t>
+          <t>~1.5 h per palletised trailer; ~3.8 h per loose container</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>&lt; 3.5 h (S023)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Picking</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pick rate</t>
+          <t>Containers unpacked inside their zone</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>order lines per picker-hour</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>% of containers whose unpacking fits the 190 m² zone</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>~56 lines/h (fast-pick 99, reserve 62, large orders 44)</t>
-        </is>
-      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>≥ 50 lines/h</t>
+          <t>91% (another 6% by lending door R2)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>≥ 90%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Picking</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Picking hours per day</t>
+          <t>Container door time</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>picker-hours, average day</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>~31 h (modelled: single-order picking, staffed for the 08:00 peak)</t>
+          <t>dock-on + unpack + palletise per 40 ft container</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>11.4 h</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>~3.3 h</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>≤ 4 h</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Picking</t>
+          <t>Inbound</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pick accuracy</t>
+          <t>Put-away cycle time</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>% of orders without a picking error</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>not in the data</t>
+          <t>minutes per pallet, reach truck</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>≥ 99.7% (scan every pick + put-to-light check)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>median 99.3%, best 99.68% (S023)</t>
+          <t>2.4 min per pallet (~25 per truck-hour)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>≤ 3 min</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Picking</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Order lead time (per order)</t>
+          <t>Pick rate</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>order received → trailer leaves</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>median 25 h, p90 102 h</t>
+          <t>order lines per picker-hour</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>median 22 h, p90 70 h</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>next day; same day if in before 12:00</t>
+          <t>~54 lines/h (fast-pick 99, reserve 49, large orders 44, small-parts shelving 50)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>≥ 50 lines/h</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Picking</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Orders shipped the same day</t>
+          <t>Fast-pick hit rate</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>% of orders</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>lines picked in the fast-pick area ÷ all picked lines</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>all orders in before 12:00</t>
+          <t>71%</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>≥ 60%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Picking</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>On-time staging</t>
+          <t>Walking per picked line</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>% of lines staged before the planned departure</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>49.9% (50.1% 'LATE', A005)</t>
+          <t>metres walked in all tours ÷ picked lines</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>≥ 98% (waves planned back from departures)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>≥ 98%</t>
+          <t>~14 m</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>≤ 15 m</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Docks</t>
+          <t>Picking</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Trailers at the doors at once</t>
+          <t>Trolley fill</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>busy day, p90</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>15 (parked all day)</t>
+          <t>volume or weight filled per trolley tour</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>max 4 of 5 doors (time slots)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>≤ 5 doors</t>
+          <t>80% (batch closed at 80%)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>75–85%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>People</t>
+          <t>Picking</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Direct labour</t>
+          <t>Small-parts picking time</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>FTE, average / peak day</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>not in the data</t>
+          <t>small-parts lines ÷ 50 lines/h</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4.7 / 8.6 FTE + 1.5 indirect</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.9 h/day for 93 lines</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>≤ 2 h/day</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>People</t>
+          <t>Picking</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Labour productivity</t>
+          <t>Picking hours per day</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>order lines per direct labour hour</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>picker-hours, average day</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>18.3 lines/h</t>
+          <t>~31 h (modelled: single-order picking, staffed for the 08:00 peak)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
+        <is>
+          <t>11.7 h</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4485,126 +5027,442 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Machinery</t>
+          <t>Picking</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Truck utilisation (average day)</t>
+          <t>Pick accuracy</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>operating h / (units × 7.5 h)</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>% of orders without a picking error</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ETV 33% · EJE 35% · ERE 14%</t>
+          <t>not in the data</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>peak day ≤ 80%</t>
+          <t>≥ 99.7% (scan every pick + put-to-light check)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>median 99.3%, best 99.68% (S023)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cost per order line</t>
+          <t>Order lead time (per order)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>(OPEX + depreciation) / lines</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>order received → trailer leaves</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>€3.78</t>
+          <t>median 25 h, p90 102 h</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>median 22 h, p90 70 h</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>p90 ≤ 72 h</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cost per order</t>
+          <t>Orders out within 24 h</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>(OPEX + depreciation) / orders</t>
+          <t>own</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>% of orders</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>€16.80</t>
+          <t>37%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>≥ 60%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>On-time shipment</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>% of lines staged before the planned departure</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>49.9% (50.1% 'LATE', A005)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>≥ 98% (every wave ends ≥ 45 min before its trailers leave)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>≥ 98%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Docks</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Trailers at the doors at once</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>busy day, p90</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>15 (parked all day)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>max 4 of 5 doors (time slots)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>≤ 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Docks</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Outbound staging fill</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>staging m² needed on the busiest afternoon ÷ 216 m²</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>46% (p90 day 28%)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>≤ 80%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Direct labour</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>FTE, average / peak day</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>not in the data</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>4.7 / 8.7 FTE + 1.5 indirect</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Labour productivity</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>order lines per direct labour hour</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>18.2 lines/h</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Machinery</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Truck utilisation (average day)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>operating h ÷ (units × 7.5 h)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>ETV 33% · EJE 31% · ERE 14%</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>peak day ≤ 80%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cost per order line</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>(OPEX + depreciation) ÷ lines</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>€3.08</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Cost per order</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>(OPEX + depreciation) ÷ orders</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>€13.68</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Safety</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Trucks and pickers separated</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>pick zones without reach-truck traffic</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>own</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>pick faces without reach-truck traffic</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>100% of pick faces (trucks refill from the rear / use perimeter + cross-aisles)</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>100% (trucks refill from the rear and use the perimeter + cross-aisles)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
         <is>
           <t>0 lost-time incidents</t>
         </is>
@@ -4621,153 +5479,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Volume</t>
+          <t>Option</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Direct FTE (peak day)</t>
+          <t>Floor m²</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>ETV 216i needed</t>
+          <t>Pallet positions used</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>EJE 120i needed</t>
+          <t>CAPEX EUR</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>ERE 225 needed</t>
+          <t>Pick rate lines/h</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Outbound doors (busiest hour)</t>
+          <t>Picking EUR/yr</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Pickers in the busiest wave</t>
+          <t>Yearly cost EUR</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>Keep in pallet racks (today)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8.6</v>
+        <v>393</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>1005</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>130650</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>49</v>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>9911</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>28576</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>one 1 m³ pallet location for a few litres of stock; long walks in the reserve aisles</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>150%</t>
+          <t>Bin shelving next to the put-wall (chosen)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>207</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>69184</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>9713</v>
       </c>
       <c r="G3" t="n">
-        <v>4</v>
+        <v>19597</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>188 bays, 2.5 m high; cheapest; fits in the packing area's spare floor; items go straight into the put-wall</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>200%</t>
+          <t>Kardex Shuttle XP 500 lifts</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>17.3</v>
+        <v>66</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>224560</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>75</v>
       </c>
       <c r="F4" t="n">
-        <v>7</v>
+        <v>6475</v>
       </c>
       <c r="G4" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>250%</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="C5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>8</v>
-      </c>
-      <c r="G5" t="n">
-        <v>7</v>
+        <v>38555</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>3 lifts ~10 m high; 3x denser, light pointer; but busy only ~6% of the day</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Explain the put-to-light wall: layout, slots, storage and worker steps
- New putwall_design.py: plan of the packing area with the 8 worker steps
  and a front view of the wall (24 x 5 = 120 tote slots, 10.8 m).
- Wall sized on totes per small order (78% one tote, 13% two, 9% 3-4):
  peak wave 73 orders x 1.35 totes x 1.2 -> 120 slots (was 90).
- D3 3.1: what the wall is, where items are stored before it, roles and
  how people move; D2 2.4 gets the figure and a short description.
- Packing-area check and CAPEX updated for the larger wall.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019BDu8Mejto8wmgVTUqspvV
</commit_message>
<xml_diff>
--- a/deliverables/Deliverable_3_Calculations.xlsx
+++ b/deliverables/Deliverable_3_Calculations.xlsx
@@ -799,10 +799,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>470905</v>
+        <v>472287</v>
       </c>
       <c r="C2" t="n">
-        <v>496225</v>
+        <v>497607</v>
       </c>
       <c r="D2" t="n">
         <v>25320</v>
@@ -815,10 +815,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>443980</v>
+        <v>445362</v>
       </c>
       <c r="C3" t="n">
-        <v>517271</v>
+        <v>518653</v>
       </c>
       <c r="D3" t="n">
         <v>73291</v>
@@ -831,10 +831,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>446129</v>
+        <v>447511</v>
       </c>
       <c r="C4" t="n">
-        <v>528920</v>
+        <v>530302</v>
       </c>
       <c r="D4" t="n">
         <v>82790</v>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>480625</v>
+        <v>482007</v>
       </c>
       <c r="C5" t="n">
-        <v>566409</v>
+        <v>567791</v>
       </c>
       <c r="D5" t="n">
         <v>85784</v>
@@ -3124,7 +3124,7 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>€3.08</t>
+          <t>€3.09</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -5422,7 +5422,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>€13.68</t>
+          <t>€13.72</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">

</xml_diff>